<commit_message>
Dashboard update 2026-08-10 14:07
</commit_message>
<xml_diff>
--- a/excel/Loanch.xlsx
+++ b/excel/Loanch.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\Loanch\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-dashboard-clean\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D57DEA6-A7C9-4BC2-A6D6-C4CE53F612F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0080911B-2B33-45E1-829A-BF243F98D892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="Z3" s="31">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.11481881737709046</v>
+        <v>0.10448089241981506</v>
       </c>
       <c r="AA3" s="29">
         <f>SUM(O3:O100)</f>
@@ -2178,11 +2178,11 @@
       </c>
       <c r="K9" s="19">
         <f ca="1">'6836f159...155f27704bef'!B12</f>
-        <v>3</v>
-      </c>
-      <c r="L9" s="19" t="str">
+        <v>-6</v>
+      </c>
+      <c r="L9" s="19">
         <f ca="1">'6836f159...155f27704bef'!P3</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="M9" s="3">
         <f>'6836f159...155f27704bef'!K3</f>
@@ -2199,7 +2199,7 @@
       <c r="P9" s="10"/>
       <c r="AC9" s="3" t="str">
         <f ca="1">'6836f159...155f27704bef'!Z3</f>
-        <v/>
+        <v>+</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.25">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="K11" s="19">
         <f ca="1">'45b52ba0...0700af8e066e'!B12</f>
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="L11" s="19" t="str">
         <f ca="1">'45b52ba0...0700af8e066e'!P3</f>
@@ -6693,7 +6693,7 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f ca="1">TODAY()</f>
-        <v>46235</v>
+        <v>46244</v>
       </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -6824,7 +6824,7 @@
         <v>36</v>
       </c>
       <c r="D3" s="11">
-        <v>46238</v>
+        <v>46261</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="19" t="str">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -9416,9 +9416,9 @@
         <f>IF(B16=K3,MAX(E:E),"")</f>
         <v/>
       </c>
-      <c r="P3" s="2" t="str">
+      <c r="P3" s="2">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
@@ -9435,7 +9435,7 @@
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
-        <v/>
+        <v>+</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>3</v>
+        <v>-6</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>

</xml_diff>